<commit_message>
Guides: the Yaoyao lessons, and the Bamboo Shard Trimmer joins The Council
Overview habits 81-83 (an edit with no effect: was its input ever found;
eliminate what before why; a shared-code fix is a change to other
characters), GameView's helper Python, same-named mods under only --from,
restore's journal and the old-vs-new-build in-game check, and Creating
Remaps START HERE rows for layered-hair shards and white cheeks.

The Council: 51 -> 52, with a credit row in the Yaoyao RemapDraft.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/YaoyaoRemapDraft.xlsx
+++ b/Data/RemapDrafts/YaoyaoRemapDraft.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +42,13 @@
       <sz val="12"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -60,17 +67,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -443,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,9 +477,17 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>🎋✂️ The Bamboo Shard Trimmer: The 52nd member of The Council</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>